<commit_message>
feat: Add RNC extraction to Mobuss scraper
- Extract RNCs linked to FVS inspections
- Store fvsId to track which FVS generated the RNC
- Export RNCs to separate Excel sheet
- Include RNC metrics in summary (count)

Structure:
- RNC contains: ID, fvsId, empreendimento, servico, descricao
- Gravidade levels: observacao, menor, maior, critica
- Status tracking: aberta, em_analise, em_correcao, em_verificacao, fechada
- Linked to FVS via fvsId field

Output:
- relatorio_mobuss.json includes rncs_extraidas array
- relatorio_mobuss.xlsx has dedicated RNCs sheet with all details
- Ready for API integration when Mobuss API becomes available

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sigq/relatorio_mobuss.xlsx
+++ b/sigq/relatorio_mobuss.xlsx
@@ -10,7 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estrutura" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campos" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opções" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RNCs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -545,24 +546,142 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Métrica</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Quantidade</t>
+          <t>FVS ID</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Empreendimento</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Servico</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Descricao</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Gravidade</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Responsavel</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Abertura</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Prazo</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>RNC-MOCK-0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>FVS-MOCK-0002</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Morada de Gaia</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Revestimento Cerâmico</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Juntas irregulares no banheiro, variacao acima do tolerado</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>em_correcao</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Construtora Alfa</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>24/04/2026</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>28/04/2026</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Métrica</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Quantidade</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>Formulários</t>
         </is>
       </c>
@@ -593,21 +712,41 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Divs</t>
+          <t>Empreendimentos</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tabelas</t>
+          <t>Servicos</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>FVS</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RNCs</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>